<commit_message>
21. Merge Two Sorted Lists
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2188CC2B-D281-478C-AC6D-2ABD3AD87E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC53E134-AE71-40EB-86BD-0500A0B6E2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -388,6 +388,14 @@
         <v>45444</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1">
+        <v>45445</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
35. Search Insert Position
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC53E134-AE71-40EB-86BD-0500A0B6E2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC079DB0-DC17-47E8-A80D-D6527DF7D728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -396,6 +396,14 @@
         <v>45445</v>
       </c>
     </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>35</v>
+      </c>
+      <c r="B5" s="1">
+        <v>45445</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
64. Minimum Path Sum
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC079DB0-DC17-47E8-A80D-D6527DF7D728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6AD46D-BB7D-47A3-A622-5B27F1B3E19E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -404,6 +404,14 @@
         <v>45445</v>
       </c>
     </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>64</v>
+      </c>
+      <c r="B6" s="1">
+        <v>45445</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
83. Remove Duplicates from Sorted List
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6AD46D-BB7D-47A3-A622-5B27F1B3E19E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930804C4-7745-4E2D-971E-99F521B91788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -412,6 +412,14 @@
         <v>45445</v>
       </c>
     </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>83</v>
+      </c>
+      <c r="B7" s="1">
+        <v>45447</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
98. Validate Binary Search Tree
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930804C4-7745-4E2D-971E-99F521B91788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{308BC86D-B1B4-49E3-9034-1101A654088F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -420,6 +420,14 @@
         <v>45447</v>
       </c>
     </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>98</v>
+      </c>
+      <c r="B8" s="1">
+        <v>45448</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
172. Factorial Trailing Zeroes
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A668CFD6-4FDA-4C9E-9E19-E182075EC9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A1B512-D013-4359-894C-DF71E8E75861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -452,6 +452,14 @@
         <v>45451</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>172</v>
+      </c>
+      <c r="B12" s="1">
+        <v>45452</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
231. Power of Two
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CCAC27C-7A70-4CA9-A403-FB22354DB1EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7332D13B-D048-4AFA-AC57-4DC862F58C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -484,6 +484,14 @@
         <v>45461</v>
       </c>
     </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A16">
+        <v>231</v>
+      </c>
+      <c r="B16" s="1">
+        <v>45461</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
342. Power of Four
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7332D13B-D048-4AFA-AC57-4DC862F58C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6517EBE-FB92-4C45-85FF-306536612A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -492,6 +492,14 @@
         <v>45461</v>
       </c>
     </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A17">
+        <v>342</v>
+      </c>
+      <c r="B17" s="1">
+        <v>45461</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
191. Number of 1 Bits
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6517EBE-FB92-4C45-85FF-306536612A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A8DF298-9B5D-4A8B-9B97-0346E1D9D688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -500,6 +500,14 @@
         <v>45461</v>
       </c>
     </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A18">
+        <v>191</v>
+      </c>
+      <c r="B18" s="1">
+        <v>45461</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
709. To Lower Case
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A8DF298-9B5D-4A8B-9B97-0346E1D9D688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D03AE30-D3C1-4CFE-B8BB-8C6D4FC25D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -508,6 +508,14 @@
         <v>45461</v>
       </c>
     </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A19">
+        <v>709</v>
+      </c>
+      <c r="B19" s="1">
+        <v>45461</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
2769. Find the Maximum Achievable Number
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D03AE30-D3C1-4CFE-B8BB-8C6D4FC25D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BE9A81-31F2-4CB0-866F-A94A72605DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -516,6 +516,14 @@
         <v>45461</v>
       </c>
     </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A20">
+        <v>2769</v>
+      </c>
+      <c r="B20" s="1">
+        <v>45464</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
3110. Score of a String
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BE9A81-31F2-4CB0-866F-A94A72605DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E356D5-78E7-4052-96CD-3ED783BD6FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -524,6 +524,14 @@
         <v>45464</v>
       </c>
     </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A21">
+        <v>3110</v>
+      </c>
+      <c r="B21" s="1">
+        <v>45464</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
326. Power of Three
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E356D5-78E7-4052-96CD-3ED783BD6FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866D9AF6-5120-41B8-B3E5-2232DE562937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -532,6 +532,14 @@
         <v>45464</v>
       </c>
     </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A22">
+        <v>326</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45464</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
1929. Concatenation of Array
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866D9AF6-5120-41B8-B3E5-2232DE562937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D916E00-BCDE-464B-A3D5-AFBF2E491196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -540,6 +540,14 @@
         <v>45464</v>
       </c>
     </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A23">
+        <v>1929</v>
+      </c>
+      <c r="B23" s="1">
+        <v>45464</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
1920. Build Array from Permutation
</commit_message>
<xml_diff>
--- a/Record.xlsx
+++ b/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benson\Desktop\Leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D916E00-BCDE-464B-A3D5-AFBF2E491196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C55EAD3-7CC8-459E-B213-5FCA2CCB6369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -548,6 +548,14 @@
         <v>45464</v>
       </c>
     </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A24">
+        <v>1920</v>
+      </c>
+      <c r="B24" s="1">
+        <v>45464</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>